<commit_message>
Add rounds 3-4 results: backup list and rejection log
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HVjeKyd47VWKq6Tz5wDcVP
</commit_message>
<xml_diff>
--- a/research/Colin_Target_Companies_Oct2026.xlsx
+++ b/research/Colin_Target_Companies_Oct2026.xlsx
@@ -8,13 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final Fits" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targets" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screened Out" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run 2 Rejected" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backup 20-49 Employees" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targets" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screened Out" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run 2 Rejected" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run 3-4 Rejected" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Targets'!$A$1:$N$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Targets'!$A$1:$N$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -686,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="25" min="1" max="1"/>
@@ -1029,12 +1031,452 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="51" t="inlineStr">
+        <is>
+          <t>Cellino</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>UNSURE</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>Cambridge, MA</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>51-200 (~80)</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>Nabiha Saklayen (co-founder/CEO)</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="inlineStr">
+        <is>
+          <t>AI/laser autonomous biomanufacturing platform for iPSC cell therapies; $80M Series A + ARPA-H up to $25M</t>
+        </is>
+      </c>
+      <c r="G8" s="27" t="inlineStr">
+        <is>
+          <t>No current sales/BD title; Chief of Staff &amp; Head of Strategy Becky Kusko was VP Head of BD 2021-23</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="inlineStr">
+        <is>
+          <t>Mostly a biotech with partnership-style deals - may not need a B2B sales motion</t>
+        </is>
+      </c>
+      <c r="I8" s="27" t="inlineStr">
+        <is>
+          <t>https://theorg.com/org/cellino/org-chart/rebecca-kusko ; https://www.zoominfo.com/c/cellino-biotech-inc/457806160</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" style="25" min="1" max="1"/>
+    <col width="22" customWidth="1" style="25" min="2" max="2"/>
+    <col width="22" customWidth="1" style="25" min="3" max="3"/>
+    <col width="30" customWidth="1" style="25" min="4" max="4"/>
+    <col width="50" customWidth="1" style="25" min="5" max="5"/>
+    <col width="55" customWidth="1" style="25" min="6" max="6"/>
+    <col width="60" customWidth="1" style="25" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="26" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C1" s="26" t="inlineStr">
+        <is>
+          <t>Employees</t>
+        </is>
+      </c>
+      <c r="D1" s="26" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="E1" s="26" t="inlineStr">
+        <is>
+          <t>What they do</t>
+        </is>
+      </c>
+      <c r="F1" s="26" t="inlineStr">
+        <is>
+          <t>Sales/BD people found</t>
+        </is>
+      </c>
+      <c r="G1" s="26" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>FemtoMetrix</t>
+        </is>
+      </c>
+      <c r="B2" s="27" t="inlineStr">
+        <is>
+          <t>Irvine, CA, USA</t>
+        </is>
+      </c>
+      <c r="C2" s="27" t="inlineStr">
+        <is>
+          <t>10-50 according to SignalHire and ZoomInfo. The exact number and whether headcount is growing are not confirmed. It could be under 20.</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>Alon Raphael (President &amp; CEO)</t>
+        </is>
+      </c>
+      <c r="E2" s="27" t="inlineStr">
+        <is>
+          <t>Optical second-harmonic-generation (SHG) inspection and metrology for non-visual defects on semiconductor wafers (Harmonic F1x system), sold to fabs.</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="inlineStr">
+        <is>
+          <t>None found. The leadership found is the CEO, CFO Tyler Rubin, CTO David Adler, EVP R&amp;D Andy Antonelli, VP Applications Kenneth James (a technical applications role, not sales), VP Engineering Timothy Wong and co-founder Hovik Nazaryan. The people listed as Directors on theorg are board members (Tom Rolfes, Charles W. Kim, Sung Hoon Yang, Wojtek Uzdelewicz). Low confidence: no sales or account-manager titles turned up, but the directories have little data on this company.</t>
+        </is>
+      </c>
+      <c r="G2" s="27" t="inlineStr">
+        <is>
+          <t>https://theorg.com/org/femtometrix ; https://theorg.com/org/femtometrix/org-chart/alon-raphael ; https://theorg.com/org/femtometrix/teams/leadership-team ; https://www.signalhire.com/companies/femtometrix-inc ; https://www.zoominfo.com/c/femtometrix-inc/363685298</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>Sepion Technologies</t>
+        </is>
+      </c>
+      <c r="B3" s="27" t="inlineStr">
+        <is>
+          <t>Emeryville, CA, USA</t>
+        </is>
+      </c>
+      <c r="C3" s="27" t="inlineStr">
+        <is>
+          <t>~24 (ZoomInfo/LeadIQ, Aug 2026); raised a $10M Series B, so not shrinking as far as I can tell</t>
+        </is>
+      </c>
+      <c r="D3" s="27" t="inlineStr">
+        <is>
+          <t>Peter Frischmann (CEO &amp; Co-Founder)</t>
+        </is>
+      </c>
+      <c r="E3" s="27" t="inlineStr">
+        <is>
+          <t>Nanoengineered separator coatings and electrolyte technology for lithium-ion and lithium-metal cell makers. It has moved from concept onto commercial production lines and won Best Commercialization Venture at the 2025 NREL Industry Growth Forum.</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="inlineStr">
+        <is>
+          <t>None found. The directory leadership is CEO Peter Frischmann, Co-Founder &amp; CSO Brett Helms, CTO Brian Sisk, VP Operations Muhammad Zahid Shafi and Director of R&amp;D Adam Ozvald. LinkedIn search showed no sales, business development or account manager staff or postings. Sales appears to be led by the CEO. Caveat: Sepion sells a coating material and process to battery manufacturers rather than equipment, so the sector fit is borderline.</t>
+        </is>
+      </c>
+      <c r="G3" s="27" t="inlineStr">
+        <is>
+          <t>https://leadiq.com/c/sepion-technologies/5e1e9ab662be9f43cad80d77/employee-directory ; https://www.zoominfo.com/pic/sepion-technologies-inc/528170000 ; https://theorg.com/org/sepion-technologies ; https://www.linkedin.com/company/sepion-technologies ; https://www.linkedin.com/in/peterfrischmann/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>SnapMagic (formerly SnapEDA)</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>San Francisco / San Mateo, CA, USA</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>About 23 (LeadIQ, Aug 2026); the largest department is engineering with 7 people</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>Natasha Baker (Founder &amp; CEO)</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Electronic component libraries (CAD symbols and footprints) and SnapMagic Copilot, an AI assistant for circuit-board designers. Its money comes mainly from electronic-component manufacturers who sponsor and promote their parts to 1.5M+ engineers.</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>No current sales leader found in any directory or LinkedIn result. LinkedIn shows an older req for a Senior Account Executive (Redwood City, $260-300K OTE, around 2024), which points to at most one senior AE. Sales looks founder-led. WEAK: the sector fit is borderline (EDA content sold to component makers' marketing teams), and I could not confirm whether the AE role was filled or whether the company is growing.</t>
+        </is>
+      </c>
+      <c r="G4" s="27" t="inlineStr">
+        <is>
+          <t>https://leadiq.com/c/snapmagic/5a1dac6b2300005e00a1ad20/employee-directory ; https://www.linkedin.com/jobs/view/senior-account-executive-at-snapmagic-3815155776 ; https://www.linkedin.com/in/natashaabaker ; https://theorg.com/org/snapeda/org-chart/natasha-baker</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Tacta Systems</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>Palo Alto, CA</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>26-45 (ZoomInfo/RocketReach range)</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>Vikram Pavate (co-founder; CEO since 2025, previously COO)</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>Tactile-sensing robotic hands plus 'Dextrous Intelligence' AI that captures skilled workers' hand data to automate high-value manufacturing tasks. Raised a $75M seed plus Series A (Matter VP, America's Frontier Fund, SBVA).</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>None found. The named team is technical: Nahid Harjee (co-founder, VP Sensing), Harry Su (Head of Robotics Engineering) and Dariusz Golda (CTO). Rafer Chambers and Monica Valadez appear in directories with roles unknown and should be confirmed.</t>
+        </is>
+      </c>
+      <c r="G5" s="27" t="inlineStr">
+        <is>
+          <t>https://rocketreach.co/tacta-systems-inc-management_b6827591c9fe6594 ; https://www.zoominfo.com/pic/tacta-systems-inc/5000066361 ; https://www.linkedin.com/in/vikram-pavate-7743884/ ; https://seedtable.com/companies/tacta-systems/funding-rounds/series-a-2025-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>HEBI Robotics</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>Pittsburgh, PA</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>11-50 per LinkedIn and ZoomInfo; exact count unverified and may be under 20</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Bob Raida (former VP Business Development and COO, now CEO)</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>Modular robotic actuators and robot-building tools sold to engineers, OEMs and industrial inspection or maintenance robot builders.</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>None besides the CEO, whose background is BD, so sales is CEO-led. Other named leaders are Dave Rollinson (CTO) and Allison Sciullo (Director of Project Management). No sales staff appeared in the directories.</t>
+        </is>
+      </c>
+      <c r="G6" s="27" t="inlineStr">
+        <is>
+          <t>https://www.therobotreport.com/hebi-robotics-promotes-raida-to-ceo-rollinson-to-cto/ ; https://rocketreach.co/hebi-robotics-management_b566cc3ef650276e ; https://www.zoominfo.com/pic/hebi-robotics/404083014 ; https://www.linkedin.com/company/hebi-robotics</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Software Defined Automation (SDA)</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>Boston, MA (stated HQ; European office in Munich, founded in Germany)</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>34 (RocketReach)</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>Josef Waltl (co-founder)</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>Industrial DevOps / software-defined PLC platform: versioning, virtualization and management of PLC and controller code across multi-vendor factories. $10M seed led by Insight Partners.</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="inlineStr">
+        <is>
+          <t>Jason Silva, 'Principal Sales Manager', per RocketReach's management list. This looks like an individual-contributor title but it was not verified in a LinkedIn result title. If he leads a team, the company fails rule 4. The real HQ (Boston or Munich) also needs confirming.</t>
+        </is>
+      </c>
+      <c r="G7" s="27" t="inlineStr">
+        <is>
+          <t>https://rocketreach.co/software-defined-automation-management_b7e9ea81c2af2227 ; https://www.linkedin.com/in/josefwaltl/ ; https://theorg.com/org/software-defined-automation?p=josef-waltl</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>Harmoni</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>~21</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>Manufacturing AI (Series A Sept 2026)</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="inlineStr">
+        <is>
+          <t>No sales leader found (failed on size only)</t>
+        </is>
+      </c>
+      <c r="G8" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>Leela AI</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>Cambridge, MA</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>~21</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>Visual AI for manufacturing operations</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="inlineStr">
+        <is>
+          <t>No sales leader found (failed on size only)</t>
+        </is>
+      </c>
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Invisible AI</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>11-50 (LinkedIn)</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Eric Danziger</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>Computer vision for manual assembly lines (Toyota)</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="inlineStr">
+        <is>
+          <t>Senior Sales Executive only; last raise 2022</t>
+        </is>
+      </c>
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/invisibleai</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1267,7 +1709,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4251,7 +4693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5231,7 +5673,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6747,4 +7189,1858 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B153"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" style="25" min="1" max="1"/>
+    <col width="110" customWidth="1" style="25" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="50" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="50" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="51" t="inlineStr">
+        <is>
+          <t>CONTINUUS Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="B2" s="27" t="inlineStr">
+        <is>
+          <t>Has an SVP, Head of Commercial (Dean Hopkins) and a Director of Business Development (Keith Barbato), plus BD associates. Directories show about 25 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="51" t="inlineStr">
+        <is>
+          <t>Cell X Technologies</t>
+        </is>
+      </c>
+      <c r="B3" s="27" t="inlineStr">
+        <is>
+          <t>Too small: 1-10 employees per directories. It also has a VP Operations who oversees sales and marketing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="51" t="inlineStr">
+        <is>
+          <t>Kytopen</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>Has a Chief Commercial Officer (Kevin Gutshall), a VP Business Development, a Senior Director of Sales and several Senior Directors of Scientific BD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="51" t="inlineStr">
+        <is>
+          <t>Akadeum Life Sciences</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>Has a VP Sales &amp; Marketing (Alexander Bukrinsky) and a VP Strategic Partnerships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="51" t="inlineStr">
+        <is>
+          <t>Quartic.ai</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>Has a Sales Director (Scott Drap, on theorg) and a second Sales Director, plus a VP Marketing. Directories show about 47 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="51" t="inlineStr">
+        <is>
+          <t>Nirrin Technologies</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>Has a Director of Sales (Evan Cooke). Directories show about 21 employees, which is below the size floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="51" t="inlineStr">
+        <is>
+          <t>LumaCyte</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>Has a President &amp; Chief Business Officer (Renee Hart, on theorg) and has had a Director of BD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="51" t="inlineStr">
+        <is>
+          <t>On Demand Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>Has a Chief Strategy and Commercial Officer. It is also mainly a drug maker (Pharmacy on Demand) rather than a tech vendor to manufacturers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="51" t="inlineStr">
+        <is>
+          <t>Title21 Health Solutions</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>Has a VP Sales &amp; Partnerships and a Director of BD. Directories show about 34 employees, based in Phoenix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="51" t="inlineStr">
+        <is>
+          <t>Invert</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>Its job post for a Life Sciences Account Executive references an existing Head of Business Development.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="51" t="inlineStr">
+        <is>
+          <t>Culture Biosciences</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>Has a built sales org: Account Director, Business Development and Senior Account Executive roles posted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="51" t="inlineStr">
+        <is>
+          <t>Pow.bio</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>Sector mismatch: its continuous fermentation is sold mainly to food and precision-fermentation customers (MeliBio honey, Bühler), not drug manufacturers. It is hiring a Senior Director of BD, and its size was not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="51" t="inlineStr">
+        <is>
+          <t>Sware (Res_Q)</t>
+        </is>
+      </c>
+      <c r="B14" s="27" t="inlineStr">
+        <is>
+          <t>Not verified, and likely has a sales team: about 69 employees and an estimated $21.6M in revenue for a SaaS company. Its sales roles could not be confirmed, so it was not passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="51" t="inlineStr">
+        <is>
+          <t>Indee Labs</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>Not verifiable: directory results mixed it up with Indee.tv, and its headcount and sales roles could not be confirmed. An Account Manager was listed. It is likely under 50 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="51" t="inlineStr">
+        <is>
+          <t>Cellular Origins</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>Headquartered in the UK (Melbourn).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="51" t="inlineStr">
+        <is>
+          <t>Artos / 83 Sciences / Tamarind Bio</t>
+        </is>
+      </c>
+      <c r="B17" s="27" t="inlineStr">
+        <is>
+          <t>Found on job boards hiring a founding AE. Out of sector: they sell R&amp;D documentation, materials discovery and drug-discovery compute, not manufacturing tech. Also likely under 20 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="51" t="inlineStr">
+        <is>
+          <t>Arena / Arena Physica (NYC, AI hardware test/verification)</t>
+        </is>
+      </c>
+      <c r="B18" s="27" t="inlineStr">
+        <is>
+          <t>Edson Greenwood leads Aerospace &amp; Defense, which is a vertical commercial leader role, and Nathan Petrie is Head of Deployment Strategy. The platform is also sold across many sectors (AMD, Bausch &amp; Lomb, defense), so it is not clearly a manufacturing-tech company. Too uncertain to pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="51" t="inlineStr">
+        <is>
+          <t>SandBox Semiconductor (Austin)</t>
+        </is>
+      </c>
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>Only about 18 employees, which is below even the near-miss floor. A LinkedIn profile titled 'Executive Business Development' (Shane Nelson) also came up in the company search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="51" t="inlineStr">
+        <is>
+          <t>Liminal (Liminal Insights, Emeryville; battery ultrasound inspection)</t>
+        </is>
+      </c>
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>Has a sales org. A LinkedIn post shows James Carrington as VP Business Development, the summary says Melissa Holler was hired as VP of Sales, and Sneha Solanki works in BD. Fails rule 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="51" t="inlineStr">
+        <is>
+          <t>Sigray (Concord CA, X-ray metrology)</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>Anasuya Adibhatla is Director, Technical Sales and Marketing (SignalHire title). A sales director (Steven Neptun) is also listed. Fails rule 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="51" t="inlineStr">
+        <is>
+          <t>Multibeam Corp (Santa Clara, e-beam lithography)</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>Has an SVP Sales &amp; Strategy, and a President (Lynn Barringer) alongside CEO David Lam. Fails rule 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="51" t="inlineStr">
+        <is>
+          <t>xLight (Palo Alto, EUV free-electron laser)</t>
+        </is>
+      </c>
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>Kevin Heidrich is listed as Chief Commercial Officer, and his LinkedIn profile came up in the xLight search. There is also a VP Global Policy &amp; Public Sector Partnerships. Fails rule 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="51" t="inlineStr">
+        <is>
+          <t>Halo Industries (Santa Clara, laser SiC wafering)</t>
+        </is>
+      </c>
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>Vinod Nair is listed as VP, Head of Sales and Marketing, and Kim Butler as a former VP Business Development. Fails rule 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="51" t="inlineStr">
+        <is>
+          <t>NovaCentrix (Austin, printed-electronics inks/photonic curing)</t>
+        </is>
+      </c>
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>Rudresh Ghosh is VP, Business &amp; Applications Development. The company is also mainly a materials/ink company. Fails rule 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="51" t="inlineStr">
+        <is>
+          <t>EUV Tech (Martinez CA, EUV metrology)</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>Christine Disbrow is Director of Business Development (her LinkedIn profile came up under EUV Tech), and Ali Husain is Director, Customer Success. Fails rule 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="51" t="inlineStr">
+        <is>
+          <t>Cetec ERP (Austin, ERP for electronics manufacturers)</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>Has a sales org: Tanner Rogers is Sales Director, plus an Executive Account Manager, an AE and an Account Manager. About 49 employees. Fails rules 4 and 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="51" t="inlineStr">
+        <is>
+          <t>Reno Sub-Systems (Reno NV, RF matching/power for fabs)</t>
+        </is>
+      </c>
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>Bill Suber is Director of Business Development. The company also has only 11-50 employees. Fails rule 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="51" t="inlineStr">
+        <is>
+          <t>SixSense</t>
+        </is>
+      </c>
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>Headquartered in Singapore, not the US.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="51" t="inlineStr">
+        <is>
+          <t>Nearfield Instruments / Delvitech / Wooptix / Invisix / AlixLabs / Galatek / Nexstrom</t>
+        </is>
+      </c>
+      <c r="B30" s="27" t="inlineStr">
+        <is>
+          <t>Not US-headquartered (Netherlands, Switzerland, Spain, EU, Sweden, China, Singapore).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="51" t="inlineStr">
+        <is>
+          <t>Substrate / Besxar</t>
+        </is>
+      </c>
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>Building their own fabs or making materials, not selling manufacturing tech to fabs. No B2B motion to build yet. Not checked further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="51" t="inlineStr">
+        <is>
+          <t>AM Batteries</t>
+        </is>
+      </c>
+      <c r="B32" s="27" t="inlineStr">
+        <is>
+          <t>Has a Chief Commercial Officer (Franz Fink), a Business Development Director (Christopher Mohajer) and a Marketing Director, per ContactOut/ZoomInfo. About 64 employees in Billerica, MA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="51" t="inlineStr">
+        <is>
+          <t>Liminal Insights</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>A search summary said Melissa Holler was appointed VP of Sales. Her name did not appear in any result title, but I rejected the company to avoid a wrong pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="51" t="inlineStr">
+        <is>
+          <t>Nanoramic Laboratories</t>
+        </is>
+      </c>
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>A CEO post advertises a Business Development Director role. The search summary also named VP Business Development holders, though not in any result title.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="51" t="inlineStr">
+        <is>
+          <t>Forge Nano</t>
+        </is>
+      </c>
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>Has a Chief Commercial Officer (Craig Steinroeder) and a Senior Sales Director, plus a sales department of about 6 people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="51" t="inlineStr">
+        <is>
+          <t>Titan Advanced Energy Solutions</t>
+        </is>
+      </c>
+      <c r="B36" s="27" t="inlineStr">
+        <is>
+          <t>Has a VP Sales &amp; Business Development (Julian Bourne). Also only 39 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="51" t="inlineStr">
+        <is>
+          <t>Sakuu</t>
+        </is>
+      </c>
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>Directory shows 4 sales staff among about 86 employees, which looks like a built sales function. No clean founder-led signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="51" t="inlineStr">
+        <is>
+          <t>Coreshell</t>
+        </is>
+      </c>
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>Directory shows 1-10 employees, below the 20-person floor even for a near-miss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="51" t="inlineStr">
+        <is>
+          <t>Citrine Informatics</t>
+        </is>
+      </c>
+      <c r="B39" s="27" t="inlineStr">
+        <is>
+          <t>Has a VP of Worldwide Sales (Rich Campbell, on theorg.com).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="51" t="inlineStr">
+        <is>
+          <t>Uncountable</t>
+        </is>
+      </c>
+      <c r="B40" s="27" t="inlineStr">
+        <is>
+          <t>Directory lists a VP Sales and a VP Sales EMEA. About 147 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="51" t="inlineStr">
+        <is>
+          <t>Modumetal</t>
+        </is>
+      </c>
+      <c r="B41" s="27" t="inlineStr">
+        <is>
+          <t>About 25 employees, down from a much larger headcount, so it fails the not-shrinking rule. It also has a Business Development Manager.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="51" t="inlineStr">
+        <is>
+          <t>actnano</t>
+        </is>
+      </c>
+      <c r="B42" s="27" t="inlineStr">
+        <is>
+          <t>Has a Global VP Sales (Jeremy Garbacik), a Head of Business Development Europe and a Sales &amp; BD Manager.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="51" t="inlineStr">
+        <is>
+          <t>Xtalic</t>
+        </is>
+      </c>
+      <c r="B43" s="27" t="inlineStr">
+        <is>
+          <t>Has a VP Business Development (John Kinne). Also only 36 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="51" t="inlineStr">
+        <is>
+          <t>MELD Manufacturing</t>
+        </is>
+      </c>
+      <c r="B44" s="27" t="inlineStr">
+        <is>
+          <t>Directory lists VPs of Sales (Louis and Jay Schlegel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="51" t="inlineStr">
+        <is>
+          <t>LiCAP Technologies</t>
+        </is>
+      </c>
+      <c r="B45" s="27" t="inlineStr">
+        <is>
+          <t>Has a VP of Sales (Marty Mills, on theorg.com) and a Sales Director.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="51" t="inlineStr">
+        <is>
+          <t>Wildcat Discovery Technologies</t>
+        </is>
+      </c>
+      <c r="B46" s="27" t="inlineStr">
+        <is>
+          <t>Has an SVP of Strategy &amp; Corporate Development (Peter Coats). It is also pivoting to making cathode material itself rather than selling technology to manufacturers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="51" t="inlineStr">
+        <is>
+          <t>VRC Metal Systems</t>
+        </is>
+      </c>
+      <c r="B47" s="27" t="inlineStr">
+        <is>
+          <t>Has a Global Business Development Manager, and a LinkedIn profile for a VP Business Development (Todd Miller) came up in the VRC search. The business is mainly aerospace and defense MRO cold spray.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="51" t="inlineStr">
+        <is>
+          <t>InfinitForm</t>
+        </is>
+      </c>
+      <c r="B48" s="27" t="inlineStr">
+        <is>
+          <t>Directory shows 1-10 employees, which is too small. It is already hiring its first AE, and a co-founder was formerly a strategic partnerships lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="51" t="inlineStr">
+        <is>
+          <t>Nox Metals</t>
+        </is>
+      </c>
+      <c r="B49" s="27" t="inlineStr">
+        <is>
+          <t>Has a Chief Revenue Officer (Kelly Gibb). Also only 1-10 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="51" t="inlineStr">
+        <is>
+          <t>Aionics</t>
+        </is>
+      </c>
+      <c r="B50" s="27" t="inlineStr">
+        <is>
+          <t>About 12 employees, too small even for a near-miss. It is an AI materials-design company.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="51" t="inlineStr">
+        <is>
+          <t>Phase3D</t>
+        </is>
+      </c>
+      <c r="B51" s="27" t="inlineStr">
+        <is>
+          <t>Directory shows 2-10 employees, which is too small.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="51" t="inlineStr">
+        <is>
+          <t>Electroninks</t>
+        </is>
+      </c>
+      <c r="B52" s="27" t="inlineStr">
+        <is>
+          <t>Has a Head of Sales &amp; Business Development (Takashi Mochizuki) and a co-founder President.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="51" t="inlineStr">
+        <is>
+          <t>3DEO</t>
+        </is>
+      </c>
+      <c r="B53" s="27" t="inlineStr">
+        <is>
+          <t>Has a Head of Sales and Business Development (Steven Rizzo) and several Business Development Reps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="51" t="inlineStr">
+        <is>
+          <t>Boston Materials</t>
+        </is>
+      </c>
+      <c r="B54" s="27" t="inlineStr">
+        <is>
+          <t>About 21 employees. It has a Director, Global Accounts and is recruiting a Director of Business Development and a Sales Manager. It also sells materials rather than process technology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="51" t="inlineStr">
+        <is>
+          <t>OneD Battery Sciences</t>
+        </is>
+      </c>
+      <c r="B55" s="27" t="inlineStr">
+        <is>
+          <t>About 40 employees and probably shrinking after it paused its Moses Lake plant plans. It previously had a Director of Sales &amp; BD, and its current commercial leadership could not be verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="51" t="inlineStr">
+        <is>
+          <t>Kelvin (kelvin.ai)</t>
+        </is>
+      </c>
+      <c r="B56" s="27" t="inlineStr">
+        <is>
+          <t>Has a Chief Business Development &amp; Strategy Officer (Sheena Chandra), which counts as a commercial C-level. Its customers are also mostly energy, oil and gas, which leans toward a sector auto-fail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="51" t="inlineStr">
+        <is>
+          <t>ProcessMiner</t>
+        </is>
+      </c>
+      <c r="B57" s="27" t="inlineStr">
+        <is>
+          <t>LinkedIn shows Rob Berman as VP of Sales (Atlanta). The company is also only about 23 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="51" t="inlineStr">
+        <is>
+          <t>Novity</t>
+        </is>
+      </c>
+      <c r="B58" s="27" t="inlineStr">
+        <is>
+          <t>theorg lists a Business Development team (Tim Curley, BD/partnerships) and a director who leads sales. Only 11-50 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="51" t="inlineStr">
+        <is>
+          <t>Arundo Analytics</t>
+        </is>
+      </c>
+      <c r="B59" s="27" t="inlineStr">
+        <is>
+          <t>theorg lists a Director of Sales (David Rogers) and a GM/VP Americas (Nick Garibay). It is mostly oil and gas, with HQ split between Oslo and Houston.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="51" t="inlineStr">
+        <is>
+          <t>TwinThread</t>
+        </is>
+      </c>
+      <c r="B60" s="27" t="inlineStr">
+        <is>
+          <t>Acquired by AVEVA in May 2026. Directories also list a VP Sales (Dave Westrom) and a CRO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="51" t="inlineStr">
+        <is>
+          <t>Plutoshift AI</t>
+        </is>
+      </c>
+      <c r="B61" s="27" t="inlineStr">
+        <is>
+          <t>theorg lists a Chief Revenue Officer (Sean Cardenas) and a Director of Customer Engagement who runs a team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="51" t="inlineStr">
+        <is>
+          <t>CVector</t>
+        </is>
+      </c>
+      <c r="B62" s="27" t="inlineStr">
+        <is>
+          <t>Only about 12 employees (TechCrunch, Jan 2026), too small even for the near-miss list. Its customers include gas utilities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="51" t="inlineStr">
+        <is>
+          <t>Ingenero</t>
+        </is>
+      </c>
+      <c r="B63" s="27" t="inlineStr">
+        <is>
+          <t>500-1,000 employees, an engineering services firm, with a VP Marketing and a business-line director.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="51" t="inlineStr">
+        <is>
+          <t>Aizon</t>
+        </is>
+      </c>
+      <c r="B64" s="27" t="inlineStr">
+        <is>
+          <t>Has a Chief Commercial Officer (Geri Studebaker), a VP of Sales and a VP of Technical Sales and Partnerships. About 155 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="51" t="inlineStr">
+        <is>
+          <t>Fuller Technologies</t>
+        </is>
+      </c>
+      <c r="B65" s="27" t="inlineStr">
+        <is>
+          <t>Large company (about 800-2,000 employees, PE-owned) with a VP and Head of Sales (Enrico Lanzini).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="51" t="inlineStr">
+        <is>
+          <t>PiControl Solutions</t>
+        </is>
+      </c>
+      <c r="B66" s="27" t="inlineStr">
+        <is>
+          <t>An old (1992) services and software firm with a Sales Manager and about 4 sales staff, under 50 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="51" t="inlineStr">
+        <is>
+          <t>Gigaton</t>
+        </is>
+      </c>
+      <c r="B67" s="27" t="inlineStr">
+        <is>
+          <t>HQ is in the UK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="51" t="inlineStr">
+        <is>
+          <t>Aimirim</t>
+        </is>
+      </c>
+      <c r="B68" s="27" t="inlineStr">
+        <is>
+          <t>HQ is not in the US (Brazil).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="51" t="inlineStr">
+        <is>
+          <t>Raven / Neuron Industries / Praxis AI / Poka Labs (YC)</t>
+        </is>
+      </c>
+      <c r="B69" s="27" t="inlineStr">
+        <is>
+          <t>Seed-stage YC companies, well under 20 employees. Poka Labs makes sales tools, not plant AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="51" t="inlineStr">
+        <is>
+          <t>Composabl</t>
+        </is>
+      </c>
+      <c r="B70" s="27" t="inlineStr">
+        <is>
+          <t>Could not verify: the search returned nothing about the company, so it was not passed. It is believed to have under 30 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="51" t="inlineStr">
+        <is>
+          <t>Vizcom</t>
+        </is>
+      </c>
+      <c r="B71" s="27" t="inlineStr">
+        <is>
+          <t>Has a Sales Director (Steve Caditz, LinkedIn) and a reported Head of Sales. It is hiring Senior Enterprise AEs and SDRs, so a sales org is being built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="51" t="inlineStr">
+        <is>
+          <t>Flexcompute</t>
+        </is>
+      </c>
+      <c r="B72" s="27" t="inlineStr">
+        <is>
+          <t>Has a Sales Director (Gowtham Krishna), plus AEs and BDRs, so the sales org is already built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="51" t="inlineStr">
+        <is>
+          <t>Luminary Cloud</t>
+        </is>
+      </c>
+      <c r="B73" s="27" t="inlineStr">
+        <is>
+          <t>A Head of Sales (Ethan Carr) is reported in RocketReach/ZoomInfo results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="51" t="inlineStr">
+        <is>
+          <t>Epsilon3</t>
+        </is>
+      </c>
+      <c r="B74" s="27" t="inlineStr">
+        <is>
+          <t>Directories list a Chief Revenue Officer (Chris Halvorsen), a Head of RevOps and 3+ AEs. It is also only 11-50 employees and aerospace-ops focused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="51" t="inlineStr">
+        <is>
+          <t>Dirac, Inc. (BuildOS)</t>
+        </is>
+      </c>
+      <c r="B75" s="27" t="inlineStr">
+        <is>
+          <t>It is scaling a GTM team with multiple AEs, a Senior AE, sales engineers and deployment strategists. It is also around 30 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="51" t="inlineStr">
+        <is>
+          <t>AllSpice</t>
+        </is>
+      </c>
+      <c r="B76" s="27" t="inlineStr">
+        <is>
+          <t>Co-founder Peter Sullivan holds the title Co-Founder &amp; Head of Growth, and it has inside sales and AE roles. It is under 50 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="51" t="inlineStr">
+        <is>
+          <t>Toolpath (Toolpath Labs, Atlanta)</t>
+        </is>
+      </c>
+      <c r="B77" s="27" t="inlineStr">
+        <is>
+          <t>Directories list a Sales Manager, a Global Account Executive and several AEs (Tony Golden, Ross Kramer, David Asbrock), so it already has 3+ AEs. It is also 11-50 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="51" t="inlineStr">
+        <is>
+          <t>Zoo (zoo.dev / KittyCAD)</t>
+        </is>
+      </c>
+      <c r="B78" s="27" t="inlineStr">
+        <is>
+          <t>A RocketReach management page lists a VP of Sales (Ian Smith). This is not fully verified, but it is too risky to pass. LinkedIn also shows only 11-50 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="51" t="inlineStr">
+        <is>
+          <t>Physna / Thangs</t>
+        </is>
+      </c>
+      <c r="B79" s="27" t="inlineStr">
+        <is>
+          <t>It has several account executives (Kevin Hoffman, Nick Thomas) and has largely moved to a consumer 3D-model marketplace (Thangs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="51" t="inlineStr">
+        <is>
+          <t>JITX</t>
+        </is>
+      </c>
+      <c r="B80" s="27" t="inlineStr">
+        <is>
+          <t>Too small: about 7-16 employees, mostly engineers. Otherwise a strong profile: CEO-led sales and hiring Founding Sales Reps in 2026. Worth revisiting once it reaches 20+.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="51" t="inlineStr">
+        <is>
+          <t>Ulendo</t>
+        </is>
+      </c>
+      <c r="B81" s="27" t="inlineStr">
+        <is>
+          <t>Too small: about 7 employees per ZoomInfo/LeadIQ. Sales is founder-led by the CEO, who builds the process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="51" t="inlineStr">
+        <is>
+          <t>Limitless Labs (LimitlessCNC)</t>
+        </is>
+      </c>
+      <c r="B82" s="27" t="inlineStr">
+        <is>
+          <t>Appears to be Israeli-founded and headquartered (Grove Ventures and Meron backing). No evidence of a US HQ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="51" t="inlineStr">
+        <is>
+          <t>Clera (simulation agent)</t>
+        </is>
+      </c>
+      <c r="B83" s="27" t="inlineStr">
+        <is>
+          <t>An early-stage SF startup hiring a Founding AE. Headcount looks far below 20 and could not be verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="51" t="inlineStr">
+        <is>
+          <t>Unravel 3D</t>
+        </is>
+      </c>
+      <c r="B84" s="27" t="inlineStr">
+        <is>
+          <t>Hiring a Founding Sales Leader, but it appears to be India-based and very early stage. No US HQ evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="51" t="inlineStr">
+        <is>
+          <t>DraftAid / REV1 / Fabricate / Jeevy (YC)</t>
+        </is>
+      </c>
+      <c r="B85" s="27" t="inlineStr">
+        <is>
+          <t>Too small (2-14 employees). DraftAid is HQ'd in Toronto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="51" t="inlineStr">
+        <is>
+          <t>Flow Engineering</t>
+        </is>
+      </c>
+      <c r="B86" s="27" t="inlineStr">
+        <is>
+          <t>HQ in London, UK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="51" t="inlineStr">
+        <is>
+          <t>Collimator</t>
+        </is>
+      </c>
+      <c r="B87" s="27" t="inlineStr">
+        <is>
+          <t>Searches returned no usable data on the company, so it is unverified and not passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="51" t="inlineStr">
+        <is>
+          <t>Formlogic (fka Subscale)</t>
+        </is>
+      </c>
+      <c r="B88" s="27" t="inlineStr">
+        <is>
+          <t>Pittsburgh software-defined precision machining manufacturer (~37 employees per directory, LinkedIn shows 51-200). Fails rule 4: contactout lists Jeffrey Wisenbaugh and Krishna Rao, both Director of Sales at Formlogic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="51" t="inlineStr">
+        <is>
+          <t>GridRaster Inc.</t>
+        </is>
+      </c>
+      <c r="B89" s="27" t="inlineStr">
+        <is>
+          <t>Mountain View industrial XR. About 34 employees, and the company is more horizontal enterprise AR/VR than manufacturing tech. Fails rule 4: directories list a Head of Enterprise Sales &amp; Strategy and Jacob Hoppen as Director of Sales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="51" t="inlineStr">
+        <is>
+          <t>Harmony AI (tryharmony.ai)</t>
+        </is>
+      </c>
+      <c r="B90" s="27" t="inlineStr">
+        <is>
+          <t>Chattanooga, TN, AI layer for factories, hiring a Founding AE, so sales is founder-led. But rocketreach shows only about 13 employees, below even the 20-employee near-miss floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="51" t="inlineStr">
+        <is>
+          <t>Laplace Robotics / Maneva</t>
+        </is>
+      </c>
+      <c r="B91" s="27" t="inlineStr">
+        <is>
+          <t>Already has a built sales org: open postings for Head of Sales, SDR, AEs and field sales reps in Atlanta, Philadelphia and Toronto (GTA). There are signs it is Canada-linked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="51" t="inlineStr">
+        <is>
+          <t>Cohesive Robotics</t>
+        </is>
+      </c>
+      <c r="B92" s="27" t="inlineStr">
+        <is>
+          <t>Brooklyn, NY welding and finishing robots, hiring a Founding AE. Only about 5 employees (1-10 per directories), far too small.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="51" t="inlineStr">
+        <is>
+          <t>Prime Robotics</t>
+        </is>
+      </c>
+      <c r="B93" s="27" t="inlineStr">
+        <is>
+          <t>Auto-fail sector: warehouse automation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="51" t="inlineStr">
+        <is>
+          <t>Dyna Robotics</t>
+        </is>
+      </c>
+      <c r="B94" s="27" t="inlineStr">
+        <is>
+          <t>Redwood City. Hired a Founding Head of Sales in 2026, and its general-purpose robot foundation models for commercial tasks (e.g., laundry and food service) fall under horizontal AI rather than manufacturing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="51" t="inlineStr">
+        <is>
+          <t>Roboto AI</t>
+        </is>
+      </c>
+      <c r="B95" s="27" t="inlineStr">
+        <is>
+          <t>Seattle, hiring a Founding AE, but it is an analytics and data platform for robotics teams in general (horizontal, not manufacturing). It is a very small seed-stage startup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="51" t="inlineStr">
+        <is>
+          <t>ChipStack</t>
+        </is>
+      </c>
+      <c r="B96" s="27" t="inlineStr">
+        <is>
+          <t>Hiring a Founding Head of Sales, but it does AI chip-design verification (EDA), which is not semiconductor manufacturing tech. Reportedly acquired by Cadence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="51" t="inlineStr">
+        <is>
+          <t>Bucket Robotics</t>
+        </is>
+      </c>
+      <c r="B97" s="27" t="inlineStr">
+        <is>
+          <t>YC S24 manufacturing vision startup, far below 20 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="51" t="inlineStr">
+        <is>
+          <t>Chemix</t>
+        </is>
+      </c>
+      <c r="B98" s="27" t="inlineStr">
+        <is>
+          <t>Sunnyvale AI-designed EV battery cells. It develops battery products rather than manufacturing tech, and its size is likely below 50. Not checked further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="51" t="inlineStr">
+        <is>
+          <t>Fexel (Forum Ventures)</t>
+        </is>
+      </c>
+      <c r="B99" s="27" t="inlineStr">
+        <is>
+          <t>Accelerator-stage industrial automation startup whose Head of Sales post is for a fractional role. Tiny, so it fails the size rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="51" t="inlineStr">
+        <is>
+          <t>FactoryFix</t>
+        </is>
+      </c>
+      <c r="B100" s="27" t="inlineStr">
+        <is>
+          <t>Recruiting/staffing platform for manufacturing trades, which is HR tech, not manufacturing tech. It also already has AEs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="51" t="inlineStr">
+        <is>
+          <t>LMI Technologies</t>
+        </is>
+      </c>
+      <c r="B101" s="27" t="inlineStr">
+        <is>
+          <t>Large established 3D inspection company (TKH Group) hiring a VP Sales, well above 250 employees, with a built sales org.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="51" t="inlineStr">
+        <is>
+          <t>Ultra Clean Technology</t>
+        </is>
+      </c>
+      <c r="B102" s="27" t="inlineStr">
+        <is>
+          <t>Large public semiconductor equipment supplier, far above 250 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="51" t="inlineStr">
+        <is>
+          <t>Slip Robotics</t>
+        </is>
+      </c>
+      <c r="B103" s="27" t="inlineStr">
+        <is>
+          <t>Already on the screened list. The job post also says the Head of Sales reports to a CRO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="51" t="inlineStr">
+        <is>
+          <t>Mindtrace</t>
+        </is>
+      </c>
+      <c r="B104" s="27" t="inlineStr">
+        <is>
+          <t>HQ is Manchester, UK, with a Detroit office. About 25 employees. Fails the US HQ rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="51" t="inlineStr">
+        <is>
+          <t>Zaimler</t>
+        </is>
+      </c>
+      <c r="B105" s="27" t="inlineStr">
+        <is>
+          <t>HQ is San Mateo, CA. It is a horizontal semantic data layer, not industrial-specific. About 12 employees. Fails on sector and size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="51" t="inlineStr">
+        <is>
+          <t>Laplace Robotics</t>
+        </is>
+      </c>
+      <c r="B106" s="27" t="inlineStr">
+        <is>
+          <t>Appears to be Canadian (madeinca.ca listing) and small. No US HQ or headcount could be confirmed, so it is not a safe pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="51" t="inlineStr">
+        <is>
+          <t>Maneva</t>
+        </is>
+      </c>
+      <c r="B107" s="27" t="inlineStr">
+        <is>
+          <t>Offices in Palo Alto and North York, Ontario. RocketReach lists April Rajchgot as Director of Enterprise Sales &amp; BD and Kevin Sun as Head of Partnerships. Fails rule 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="51" t="inlineStr">
+        <is>
+          <t>Hellbender</t>
+        </is>
+      </c>
+      <c r="B108" s="27" t="inlineStr">
+        <is>
+          <t>Pittsburgh, about 94 employees. Directories list Ty Fraley (Head of BD), Brett Phillips (Chief Business Development Officer) and David Tusick (Chief Growth Officer). Its products also target retail and fleet use. Fails rule 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="51" t="inlineStr">
+        <is>
+          <t>Shelfmark</t>
+        </is>
+      </c>
+      <c r="B109" s="27" t="inlineStr">
+        <is>
+          <t>Pittsburgh, about 16 employees. Ron Gabriel is Head of Business Development. Too small for a near-miss and fails rule 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="51" t="inlineStr">
+        <is>
+          <t>Cerrion</t>
+        </is>
+      </c>
+      <c r="B110" s="27" t="inlineStr">
+        <is>
+          <t>HQ is Zurich, Switzerland (11-50 employees). It is hiring a founding US AE but is not US-headquartered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="51" t="inlineStr">
+        <is>
+          <t>OpenBOM</t>
+        </is>
+      </c>
+      <c r="B111" s="27" t="inlineStr">
+        <is>
+          <t>About 14 employees. RocketReach lists Mark Gartner as CRO plus an AE, a Sales Ops lead and an SDR. Fails rules 3, 4 and 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="51" t="inlineStr">
+        <is>
+          <t>1872</t>
+        </is>
+      </c>
+      <c r="B112" s="27" t="inlineStr">
+        <is>
+          <t>Cincinnati, AI-native steel fabrication. Only 9 employees, and it serves construction, energy and utility customers. Fails on size and sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="51" t="inlineStr">
+        <is>
+          <t>Ohm (YC W23)</t>
+        </is>
+      </c>
+      <c r="B113" s="27" t="inlineStr">
+        <is>
+          <t>San Francisco, 7 employees. Too small.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="51" t="inlineStr">
+        <is>
+          <t>Xact Metal</t>
+        </is>
+      </c>
+      <c r="B114" s="27" t="inlineStr">
+        <is>
+          <t>Has a VP Global Sales (Mark Barfoot), a VP NA Sales &amp; Partnerships and several Senior Sales Managers. Fails rules 4 and 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="51" t="inlineStr">
+        <is>
+          <t>Haven Safety AI</t>
+        </is>
+      </c>
+      <c r="B115" s="27" t="inlineStr">
+        <is>
+          <t>San Francisco, a small AI Fund/AES spinout. Horizontal EHS software for energy, construction and logistics. Fails on sector and size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="51" t="inlineStr">
+        <is>
+          <t>CADDi</t>
+        </is>
+      </c>
+      <c r="B116" s="27" t="inlineStr">
+        <is>
+          <t>Chicago US arm, about 367 employees, with multiple Mid-Market and Enterprise AE openings. Fails on size and sales org.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="51" t="inlineStr">
+        <is>
+          <t>Fexel</t>
+        </is>
+      </c>
+      <c r="B117" s="27" t="inlineStr">
+        <is>
+          <t>Forum Ventures studio company hiring a fractional Head of Sales. Very early stage and almost certainly under 20 employees. Not verified further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="51" t="inlineStr">
+        <is>
+          <t>Foundation EGI</t>
+        </is>
+      </c>
+      <c r="B118" s="27" t="inlineStr">
+        <is>
+          <t>Already screened, listed as Foundation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="51" t="inlineStr">
+        <is>
+          <t>Saphira AI / Paragon AI / Metaprise</t>
+        </is>
+      </c>
+      <c r="B119" s="27" t="inlineStr">
+        <is>
+          <t>YC/seed-stage companies with founding AE postings. Likely under 20 employees, and Metaprise and Paragon are not clearly industrial. Not verified because of the search budget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="51" t="inlineStr">
+        <is>
+          <t>ECM PCB Stator Tech</t>
+        </is>
+      </c>
+      <c r="B120" s="27" t="inlineStr">
+        <is>
+          <t>Has an EVP of Global Sales and Marketing (Michael Fischer). Also only 11-50 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="51" t="inlineStr">
+        <is>
+          <t>SiLC Technologies</t>
+        </is>
+      </c>
+      <c r="B121" s="27" t="inlineStr">
+        <is>
+          <t>Has a VP of Business Development and Marketing (Ralf Muenster) and a VP of Market Development (Arlon Martin).</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="51" t="inlineStr">
+        <is>
+          <t>Voyant Photonics</t>
+        </is>
+      </c>
+      <c r="B122" s="27" t="inlineStr">
+        <is>
+          <t>Has a Senior Director of Sales &amp; BD (Stephen Miller) and a Sales Director Europe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="51" t="inlineStr">
+        <is>
+          <t>Bedrock Automation</t>
+        </is>
+      </c>
+      <c r="B123" s="27" t="inlineStr">
+        <is>
+          <t>Shut down in 2022 after the ADI/Maxim merger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="51" t="inlineStr">
+        <is>
+          <t>Cirrus Link Solutions</t>
+        </is>
+      </c>
+      <c r="B124" s="27" t="inlineStr">
+        <is>
+          <t>Only 2-10 employees on LinkedIn, too small even for a near-miss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="51" t="inlineStr">
+        <is>
+          <t>Linear Labs</t>
+        </is>
+      </c>
+      <c r="B125" s="27" t="inlineStr">
+        <is>
+          <t>No sales leader found (CEO Brad Hunstable, CTO Fred Hunstable, VP Engineering Erik Hatch). But headcount is unverified (11-50, about $1M revenue, possibly under 20), and the motors are aimed mainly at EVs/HVAC, so the sector is borderline. Not confident enough to list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="51" t="inlineStr">
+        <is>
+          <t>Adaptive Machines</t>
+        </is>
+      </c>
+      <c r="B126" s="27" t="inlineStr">
+        <is>
+          <t>Could not confirm size or leadership in directories (founder possibly David Braun). Looks very early stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="51" t="inlineStr">
+        <is>
+          <t>Automat</t>
+        </is>
+      </c>
+      <c r="B127" s="27" t="inlineStr">
+        <is>
+          <t>Hiring a Head of Sales, but HQ, sector and size were not checked within the search budget. Not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="51" t="inlineStr">
+        <is>
+          <t>Ohm / Saphira AI / Cerrion / Pendulum Robotics (YC)</t>
+        </is>
+      </c>
+      <c r="B128" s="27" t="inlineStr">
+        <is>
+          <t>Seen in founding-AE job searches. YC hardware startups are likely under 20 employees, and Cerrion is Swiss. Not pursued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="51" t="inlineStr">
+        <is>
+          <t>MarqMetrix</t>
+        </is>
+      </c>
+      <c r="B129" s="27" t="inlineStr">
+        <is>
+          <t>Now part of Thermo Fisher Scientific (LinkedIn company page 'MarqMetrix, part of Thermo Fisher Scientific'). Not independent, and it had a Sales Director.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="51" t="inlineStr">
+        <is>
+          <t>Creative Electron</t>
+        </is>
+      </c>
+      <c r="B130" s="27" t="inlineStr">
+        <is>
+          <t>Has a built sales org: Troy Johnson, Sales Manager North America; Giancarlo de la Garza, Business Unit Director over sales; plus technical sales staff (Carlos Valenzuela, Alex Monge).</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="51" t="inlineStr">
+        <is>
+          <t>Revel (Revel Software Corp, LA)</t>
+        </is>
+      </c>
+      <c r="B131" s="27" t="inlineStr">
+        <is>
+          <t>11-50 employees and a $1B+ valuation after a $150M Series B (Feb 2026). Its job post describes an existing 'enterprise sales organization'. Customers are mostly aerospace, defense, space and nuclear, not manufacturers. Not a fractional-CRO buyer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="51" t="inlineStr">
+        <is>
+          <t>HyperSpectral Corp (Alexandria, VA)</t>
+        </is>
+      </c>
+      <c r="B132" s="27" t="inlineStr">
+        <is>
+          <t>Sector does not fit: AI spectral particle detection is not clearly sold to manufacturers. Small Series A company. Not pursued further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="51" t="inlineStr">
+        <is>
+          <t>Fractilia (Austin, TX)</t>
+        </is>
+      </c>
+      <c r="B133" s="27" t="inlineStr">
+        <is>
+          <t>Fits the sector (semiconductor stochastics metrology software) and shows no VP Sales, but headcount looks well under 20 and I could not confirm it. Sales appears to run through contracted 'Business Consultants' (Terry Skales, Mike Kirk). Too small, unverified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="51" t="inlineStr">
+        <is>
+          <t>Verisurf Software</t>
+        </is>
+      </c>
+      <c r="B134" s="27" t="inlineStr">
+        <is>
+          <t>Pat Bass is Director of Sales, David Olson is Director of Sales and Marketing, plus a Sales Manager and a Global BD Manager. The sales department has about 15 people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="51" t="inlineStr">
+        <is>
+          <t>Applied Vision Corporation (Antares Vision Group - Rigid Containers)</t>
+        </is>
+      </c>
+      <c r="B135" s="27" t="inlineStr">
+        <is>
+          <t>Owned by Antares Vision. Jeff Hartung is VP Sales, Darren Hench is VP Key Accounts, plus regional sales directors and managers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="51" t="inlineStr">
+        <is>
+          <t>Xallent (Ithaca, NY)</t>
+        </is>
+      </c>
+      <c r="B136" s="27" t="inlineStr">
+        <is>
+          <t>Too small: about 463 LinkedIn followers, well under 20 employees. No size-only near-miss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="51" t="inlineStr">
+        <is>
+          <t>Machine Vision Products Inc (Carlsbad, CA)</t>
+        </is>
+      </c>
+      <c r="B137" s="27" t="inlineStr">
+        <is>
+          <t>Paul Groome is Director of Sales and Support, Danny Tan is Sales Manager SEA, and Antoine Ayoub is Enterprise Account Manager.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="51" t="inlineStr">
+        <is>
+          <t>Hundred (YC)</t>
+        </is>
+      </c>
+      <c r="B138" s="27" t="inlineStr">
+        <is>
+          <t>Early-stage YC inspection startup, far below 20 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="51" t="inlineStr">
+        <is>
+          <t>Coherix (Ann Arbor, MI)</t>
+        </is>
+      </c>
+      <c r="B139" s="27" t="inlineStr">
+        <is>
+          <t>Two VPs of Business Development (Mark McCarthy, Hollis McNully), a Global Director of Sales (David Stott), a Director of New BD and account managers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="51" t="inlineStr">
+        <is>
+          <t>Erbessd Instruments (Glens Falls, NY)</t>
+        </is>
+      </c>
+      <c r="B140" s="27" t="inlineStr">
+        <is>
+          <t>The CEO also holds the title EVP Global Sales and Distribution. Regional sales managers (LATAM, distributor), inside sales staff and a sales operations admin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="51" t="inlineStr">
+        <is>
+          <t>TiHive</t>
+        </is>
+      </c>
+      <c r="B141" s="27" t="inlineStr">
+        <is>
+          <t>HQ in France (Grenoble), not the US.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="51" t="inlineStr">
+        <is>
+          <t>Intenseye</t>
+        </is>
+      </c>
+      <c r="B142" s="27" t="inlineStr">
+        <is>
+          <t>Sector is EHS/workplace-safety vision, which is horizontal, and it already has a built sales org.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="51" t="inlineStr">
+        <is>
+          <t>Polaris Automation, Inc. (Columbus, OH; Chordata MES)</t>
+        </is>
+      </c>
+      <c r="B143" s="27" t="inlineStr">
+        <is>
+          <t>Fails rules 4 and 5. Directory results (RocketReach/ZoomInfo) list several Sales Directors (Randy Mingee, Derek Simonette and others), Senior Account Managers and a Director of Sales Operations. It also mixes product with integrator services. Founded in 1984, 51-200 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="51" t="inlineStr">
+        <is>
+          <t>StartProto (Atlanta, GA)</t>
+        </is>
+      </c>
+      <c r="B144" s="27" t="inlineStr">
+        <is>
+          <t>Too small. LinkedIn shows 2-10 employees (about 17 visible), below even the near-miss floor. It is hiring a Founding AE, so sales is founder-led.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="51" t="inlineStr">
+        <is>
+          <t>Acerta Analytics</t>
+        </is>
+      </c>
+      <c r="B145" s="27" t="inlineStr">
+        <is>
+          <t>HQ is Kitchener, Ontario, Canada, with 11-50 employees. A Detroit-based Founding AE job ad does not change where the company is headquartered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="51" t="inlineStr">
+        <is>
+          <t>Cohesive Robotics (Brooklyn, NY)</t>
+        </is>
+      </c>
+      <c r="B146" s="27" t="inlineStr">
+        <is>
+          <t>Too small: 2-10 employees on LinkedIn. It is hiring a Founding AE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="51" t="inlineStr">
+        <is>
+          <t>Datanomix (Nashua, NH)</t>
+        </is>
+      </c>
+      <c r="B147" s="27" t="inlineStr">
+        <is>
+          <t>Fails rule 5 and the size rule. It has a built sales org: several AEs (Andrew Lusty, Brendan Walsh and others), Senior BD leads and BDRs, with a VP of Customer Success over a sales department of about 14. It has 11-50 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="51" t="inlineStr">
+        <is>
+          <t>PickNik Robotics (Boulder, CO)</t>
+        </is>
+      </c>
+      <c r="B148" s="27" t="inlineStr">
+        <is>
+          <t>Has a Director of Business Development (Sean Kolk, per LinkedIn) and a CEO with an enterprise sales background. Reportedly acquired by Qualcomm. Its robotics software is horizontal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="51" t="inlineStr">
+        <is>
+          <t>Loopr AI (Seattle, WA)</t>
+        </is>
+      </c>
+      <c r="B149" s="27" t="inlineStr">
+        <is>
+          <t>Has a Sales Director (a company post welcomed Monica Lazo as Sales Director). About 20+ employees, so too small anyway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="51" t="inlineStr">
+        <is>
+          <t>1872 (Cincinnati, OH)</t>
+        </is>
+      </c>
+      <c r="B150" s="27" t="inlineStr">
+        <is>
+          <t>Seed-stage (raised $15M) autonomous structural-steel fabrication factory, so its customers are in construction (an auto-fail sector). Headcount looks well under 20, mostly fabrication techs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="51" t="inlineStr">
+        <is>
+          <t>Shelfmark (Pittsburgh, PA)</t>
+        </is>
+      </c>
+      <c r="B151" s="27" t="inlineStr">
+        <is>
+          <t>Wrong sector: retail shelf-inventory AI (deployed at 7-Eleven). It has 2-10 employees and a Head of Business Development.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="51" t="inlineStr">
+        <is>
+          <t>Fexel (Chicago Heights, IL)</t>
+        </is>
+      </c>
+      <c r="B152" s="27" t="inlineStr">
+        <is>
+          <t>Not verified because the search budget ran out. It is a very early-stage industrial automation startup posting a fractional Head of Sales and is likely under 20 employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="51" t="inlineStr">
+        <is>
+          <t>Midwest Engineered Systems / HS Inc. Automation / Axis Company</t>
+        </is>
+      </c>
+      <c r="B153" s="27" t="inlineStr">
+        <is>
+          <t>Not checked. These are traditional robotics integrators (custom machine builders) without a scalable product, and they typically have established sales or estimating teams.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>